<commit_message>
Sprint 3 sprint planning files
</commit_message>
<xml_diff>
--- a/capstone/sprint3/26-10-sprint-3-initial-metrics.xlsx
+++ b/capstone/sprint3/26-10-sprint-3-initial-metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\styne\Lewis\software\Stone-Ocean-Backlogs\capstone\sprint3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95738EEB-4692-4DAF-8950-1488BDFDB332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7952B809-4483-4993-B9F3-5EDF4300770A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="44">
   <si>
     <t>Name</t>
   </si>
@@ -164,6 +164,15 @@
   </si>
   <si>
     <t xml:space="preserve">Juno Tyne </t>
+  </si>
+  <si>
+    <t>JT</t>
+  </si>
+  <si>
+    <t>9/22/2026 11:56am</t>
+  </si>
+  <si>
+    <t>RW</t>
   </si>
 </sst>
 </file>
@@ -37127,7 +37136,9 @@
       <c r="B9" s="7">
         <v>10</v>
       </c>
-      <c r="C9" s="7"/>
+      <c r="C9" s="7">
+        <v>9</v>
+      </c>
       <c r="D9" s="7"/>
       <c r="E9" s="7"/>
       <c r="F9" s="8"/>
@@ -37135,9 +37146,9 @@
         <f t="shared" ref="G9:H12" si="0">D9/B9</f>
         <v>0</v>
       </c>
-      <c r="H9" s="10" t="e">
+      <c r="H9" s="10">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="I9" s="10">
         <f t="shared" ref="I9:I16" si="1">E9/B9</f>
@@ -37151,7 +37162,9 @@
       <c r="B10" s="7">
         <v>12</v>
       </c>
-      <c r="C10" s="7"/>
+      <c r="C10" s="7">
+        <v>14</v>
+      </c>
       <c r="D10" s="7"/>
       <c r="E10" s="7"/>
       <c r="F10" s="8"/>
@@ -37159,9 +37172,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H10" s="10" t="e">
+      <c r="H10" s="10">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="I10" s="10">
         <f t="shared" si="1"/>
@@ -37175,7 +37188,9 @@
       <c r="B11" s="7">
         <v>12</v>
       </c>
-      <c r="C11" s="7"/>
+      <c r="C11" s="7">
+        <v>12</v>
+      </c>
       <c r="D11" s="7"/>
       <c r="E11" s="7"/>
       <c r="F11" s="8"/>
@@ -37183,9 +37198,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H11" s="10" t="e">
+      <c r="H11" s="10">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="I11" s="10">
         <f t="shared" si="1"/>
@@ -37199,7 +37214,9 @@
       <c r="B12" s="7">
         <v>12</v>
       </c>
-      <c r="C12" s="7"/>
+      <c r="C12" s="7">
+        <v>13</v>
+      </c>
       <c r="D12" s="7"/>
       <c r="E12" s="7"/>
       <c r="F12" s="8"/>
@@ -37207,9 +37224,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H12" s="10" t="e">
+      <c r="H12" s="10">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="I12" s="10">
         <f t="shared" si="1"/>
@@ -37259,7 +37276,7 @@
       </c>
       <c r="C16" s="7">
         <f>SUM(C9:C14)</f>
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="D16" s="7">
         <f>SUM(D9:D14)</f>
@@ -37274,9 +37291,9 @@
         <f t="shared" ref="G16:H16" si="2">D16/B16</f>
         <v>0</v>
       </c>
-      <c r="H16" s="10" t="e">
+      <c r="H16" s="10">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="I16" s="10">
         <f t="shared" si="1"/>
@@ -37312,18 +37329,26 @@
       <c r="A20" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="16"/>
+      <c r="B20" s="16" t="s">
+        <v>41</v>
+      </c>
       <c r="C20" s="16"/>
-      <c r="D20" s="17"/>
+      <c r="D20" s="17" t="s">
+        <v>42</v>
+      </c>
       <c r="E20" s="3"/>
     </row>
     <row r="21" spans="1:9" ht="15.75" customHeight="1">
       <c r="A21" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B21" s="10"/>
+      <c r="B21" s="10" t="s">
+        <v>43</v>
+      </c>
       <c r="C21" s="16"/>
-      <c r="D21" s="17"/>
+      <c r="D21" s="17">
+        <v>46288.497916666667</v>
+      </c>
       <c r="E21" s="7"/>
     </row>
     <row r="22" spans="1:9" ht="15.75" customHeight="1">

</xml_diff>